<commit_message>
Corregir: lote cortado son UND de producción, no restan inventario kg
El lote Mar Kids (1.300 und) usó tela WIP en planta. Solo descuenta
unidades de la meta Mar KIDS; el inventario de la foto se usa completo.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/PLAN_PRIORIDADES_MAR_RIO_KIDS.xlsx
+++ b/output/PLAN_PRIORIDADES_MAR_RIO_KIDS.xlsx
@@ -495,41 +495,43 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tela usada lote Mar Kids cortado (kg)</t>
+          <t>Inventario tela actual (kg) — foto</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>338</v>
+        <v>2991.18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tela neta (kg)</t>
+          <t>Lote Mar Kids cortado (und) — tela de PRODUCCIÓN, no inventario</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2777.93</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Lote Mar Kids cortado (und)</t>
+          <t>Und/color lote (~118 und, rep. proporcional)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1300</v>
+        <v>118.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Und/color lote (~)</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>118.2</v>
+          <t>Nota lote</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Solo descuenta UND de meta Mar KIDS; NO resta kg del inventario</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -681,17 +683,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -702,35 +703,30 @@
       </c>
       <c r="B1" s="3" t="inlineStr">
         <is>
-          <t>Stock kg</t>
+          <t>Inventario kg (foto)</t>
         </is>
       </c>
       <c r="C1" s="3" t="inlineStr">
         <is>
-          <t>Usado lote Mar Kids</t>
+          <t>Und ya cortadas Mar KIDS</t>
         </is>
       </c>
       <c r="D1" s="3" t="inlineStr">
         <is>
-          <t>Neto kg</t>
+          <t>Max und Mar KIDS Excel</t>
         </is>
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Max und Mar KIDS</t>
+          <t>Max und Rio KIDS</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
         <is>
-          <t>Max und Rio KIDS</t>
+          <t>Max und Mar CAB</t>
         </is>
       </c>
       <c r="G1" s="3" t="inlineStr">
-        <is>
-          <t>Max und Mar CAB</t>
-        </is>
-      </c>
-      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Alerta</t>
         </is>
@@ -746,21 +742,18 @@
         <v>689.9</v>
       </c>
       <c r="C2" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D2" t="n">
-        <v>659.17</v>
+        <v>409</v>
       </c>
       <c r="E2" t="n">
-        <v>409</v>
+        <v>361</v>
       </c>
       <c r="F2" t="n">
-        <v>361</v>
-      </c>
-      <c r="G2" t="n">
         <v>473</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>ALTA flexibilidad</t>
         </is>
@@ -776,21 +769,18 @@
         <v>657.16</v>
       </c>
       <c r="C3" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D3" t="n">
-        <v>626.4299999999999</v>
+        <v>379</v>
       </c>
       <c r="E3" t="n">
-        <v>379</v>
+        <v>317</v>
       </c>
       <c r="F3" t="n">
-        <v>317</v>
-      </c>
-      <c r="G3" t="n">
         <v>555</v>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>ALTA flexibilidad</t>
         </is>
@@ -806,21 +796,18 @@
         <v>348.34</v>
       </c>
       <c r="C4" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D4" t="n">
-        <v>317.61</v>
+        <v>243</v>
       </c>
       <c r="E4" t="n">
-        <v>243</v>
+        <v>215</v>
       </c>
       <c r="F4" t="n">
-        <v>215</v>
-      </c>
-      <c r="G4" t="n">
         <v>151</v>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -836,21 +823,18 @@
         <v>271.46</v>
       </c>
       <c r="C5" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D5" t="n">
-        <v>240.73</v>
+        <v>232</v>
       </c>
       <c r="E5" t="n">
-        <v>232</v>
+        <v>284</v>
       </c>
       <c r="F5" t="n">
-        <v>284</v>
-      </c>
-      <c r="G5" t="n">
         <v>205</v>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -866,21 +850,18 @@
         <v>221</v>
       </c>
       <c r="C6" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D6" t="n">
-        <v>190.27</v>
+        <v>153</v>
       </c>
       <c r="E6" t="n">
-        <v>153</v>
+        <v>351</v>
       </c>
       <c r="F6" t="n">
-        <v>351</v>
-      </c>
-      <c r="G6" t="n">
         <v>268</v>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -896,21 +877,18 @@
         <v>188.44</v>
       </c>
       <c r="C7" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D7" t="n">
-        <v>157.71</v>
+        <v>254</v>
       </c>
       <c r="E7" t="n">
-        <v>254</v>
+        <v>294</v>
       </c>
       <c r="F7" t="n">
-        <v>294</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="inlineStr">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -926,21 +904,18 @@
         <v>175.38</v>
       </c>
       <c r="C8" t="n">
-        <v>30.73</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>144.65</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" t="n">
         <v>124</v>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -959,18 +934,15 @@
         <v>0</v>
       </c>
       <c r="D9" t="n">
-        <v>162.04</v>
+        <v>460</v>
       </c>
       <c r="E9" t="n">
-        <v>460</v>
+        <v>224</v>
       </c>
       <c r="F9" t="n">
-        <v>224</v>
-      </c>
-      <c r="G9" t="n">
         <v>390</v>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -989,7 +961,7 @@
         <v>0</v>
       </c>
       <c r="D10" t="n">
-        <v>94.2</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
@@ -997,10 +969,7 @@
       <c r="F10" t="n">
         <v>0</v>
       </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -1019,18 +988,15 @@
         <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>57.94</v>
+        <v>114</v>
       </c>
       <c r="E11" t="n">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="F11" t="n">
-        <v>130</v>
-      </c>
-      <c r="G11" t="n">
         <v>67</v>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>MEDIA</t>
         </is>
@@ -1046,23 +1012,20 @@
         <v>47.68</v>
       </c>
       <c r="C12" t="n">
-        <v>30.73</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>16.95</v>
+        <v>0</v>
       </c>
       <c r="E12" t="n">
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
         <v>190</v>
       </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>BAJA</t>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
     </row>
@@ -1076,23 +1039,20 @@
         <v>46.02</v>
       </c>
       <c r="C13" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D13" t="n">
-        <v>15.29</v>
+        <v>224</v>
       </c>
       <c r="E13" t="n">
-        <v>224</v>
+        <v>162</v>
       </c>
       <c r="F13" t="n">
-        <v>162</v>
-      </c>
-      <c r="G13" t="n">
         <v>355</v>
       </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>BAJA</t>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
     </row>
@@ -1106,23 +1066,20 @@
         <v>31.44</v>
       </c>
       <c r="C14" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D14" t="n">
-        <v>0.71</v>
+        <v>214</v>
       </c>
       <c r="E14" t="n">
-        <v>214</v>
+        <v>142</v>
       </c>
       <c r="F14" t="n">
-        <v>142</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>BAJA</t>
+        <v>0</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>MEDIA</t>
         </is>
       </c>
     </row>
@@ -1136,51 +1093,18 @@
         <v>0.18</v>
       </c>
       <c r="C15" t="n">
-        <v>30.73</v>
+        <v>118.2</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>239</v>
       </c>
       <c r="E15" t="n">
-        <v>239</v>
+        <v>260</v>
       </c>
       <c r="F15" t="n">
-        <v>260</v>
-      </c>
-      <c r="G15" t="n">
         <v>122</v>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>SIN STOCK</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Púrpura</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="n">
-        <v>180</v>
-      </c>
-      <c r="F16" t="n">
-        <v>212</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>SIN STOCK</t>
         </is>
@@ -1304,7 +1228,7 @@
         <v>145</v>
       </c>
       <c r="G3" t="n">
-        <v>659.17</v>
+        <v>689.9</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -1334,7 +1258,7 @@
         <v>130</v>
       </c>
       <c r="G4" t="n">
-        <v>626.4299999999999</v>
+        <v>657.16</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1364,7 +1288,7 @@
         <v>67</v>
       </c>
       <c r="G5" t="n">
-        <v>157.71</v>
+        <v>188.44</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1394,7 +1318,7 @@
         <v>62</v>
       </c>
       <c r="G6" t="n">
-        <v>317.61</v>
+        <v>348.34</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1424,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1454,7 +1378,7 @@
         <v>56</v>
       </c>
       <c r="G8" t="n">
-        <v>240.73</v>
+        <v>271.46</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1484,7 +1408,7 @@
         <v>52</v>
       </c>
       <c r="G9" t="n">
-        <v>15.29</v>
+        <v>46.02</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1511,14 +1435,14 @@
         <v>47</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="G10" t="n">
-        <v>0.71</v>
+        <v>31.44</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -1574,7 +1498,7 @@
         <v>17</v>
       </c>
       <c r="G12" t="n">
-        <v>190.27</v>
+        <v>221</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1777,7 +1701,7 @@
         <v>0.26</v>
       </c>
       <c r="N2" s="4" t="n">
-        <v>301.49</v>
+        <v>332.22</v>
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
@@ -1897,7 +1821,7 @@
         <v>0.26</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>185.85</v>
+        <v>216.58</v>
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
@@ -1957,7 +1881,7 @@
         <v>0.26</v>
       </c>
       <c r="N5" s="4" t="n">
-        <v>621.47</v>
+        <v>652.2</v>
       </c>
       <c r="O5" s="4" t="inlineStr">
         <is>
@@ -2021,7 +1945,7 @@
         <v>0.26</v>
       </c>
       <c r="N6" s="4" t="n">
-        <v>226.17</v>
+        <v>256.9</v>
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
@@ -2141,7 +2065,7 @@
         <v>0.26</v>
       </c>
       <c r="N8" s="4" t="n">
-        <v>140.29</v>
+        <v>171.02</v>
       </c>
       <c r="O8" s="4" t="inlineStr">
         <is>
@@ -2201,7 +2125,7 @@
         <v>0.26</v>
       </c>
       <c r="N9" s="4" t="n">
-        <v>592.63</v>
+        <v>623.36</v>
       </c>
       <c r="O9" s="4" t="inlineStr">
         <is>
@@ -2325,7 +2249,7 @@
         <v>0.26</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O11" s="4" t="inlineStr">
         <is>
@@ -2380,27 +2304,23 @@
         <v>47</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>0</v>
+        <v>12.22</v>
       </c>
       <c r="M12" s="4" t="n">
         <v>0.26</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>0.71</v>
+        <v>19.22</v>
       </c>
       <c r="O12" s="4" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
-        </is>
-      </c>
-      <c r="P12" s="4" t="inlineStr">
-        <is>
-          <t>Stock crítico — excluir o esperar compra</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
@@ -2453,7 +2373,7 @@
         <v>0.26</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>1.77</v>
+        <v>32.5</v>
       </c>
       <c r="O13" s="4" t="inlineStr">
         <is>
@@ -2513,7 +2433,7 @@
         <v>0.32</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>267.25</v>
+        <v>297.98</v>
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
@@ -2633,7 +2553,7 @@
         <v>0.32</v>
       </c>
       <c r="N16" s="4" t="n">
-        <v>129.85</v>
+        <v>160.58</v>
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
@@ -2693,7 +2613,7 @@
         <v>0.32</v>
       </c>
       <c r="N17" s="4" t="n">
-        <v>563.87</v>
+        <v>594.6</v>
       </c>
       <c r="O17" s="4" t="inlineStr">
         <is>
@@ -2757,7 +2677,7 @@
         <v>0.32</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>180.73</v>
+        <v>211.46</v>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
@@ -2877,7 +2797,7 @@
         <v>0.32</v>
       </c>
       <c r="N20" s="4" t="n">
-        <v>93.25</v>
+        <v>123.98</v>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
@@ -2937,7 +2857,7 @@
         <v>0.32</v>
       </c>
       <c r="N21" s="4" t="n">
-        <v>542.0700000000001</v>
+        <v>572.8</v>
       </c>
       <c r="O21" s="4" t="inlineStr">
         <is>
@@ -3061,7 +2981,7 @@
         <v>0.32</v>
       </c>
       <c r="N23" s="4" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
@@ -3116,27 +3036,23 @@
         <v>71</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>0</v>
+        <v>19.2</v>
       </c>
       <c r="M24" s="4" t="n">
         <v>0.32</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>0.71</v>
+        <v>0.02</v>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="inlineStr">
-        <is>
-          <t>Stock crítico — excluir o esperar compra</t>
-        </is>
-      </c>
+          <t>PARCIAL (limitado tela)</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n">
@@ -3180,27 +3096,23 @@
         <v>81</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="L25" s="4" t="n">
-        <v>0</v>
+        <v>25.92</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>0.32</v>
       </c>
       <c r="N25" s="4" t="n">
-        <v>1.77</v>
+        <v>6.58</v>
       </c>
       <c r="O25" s="4" t="inlineStr">
         <is>
-          <t>PARCIAL (limitado tela)</t>
-        </is>
-      </c>
-      <c r="P25" s="4" t="inlineStr">
-        <is>
-          <t>Limitado por tela disponible</t>
-        </is>
-      </c>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="P25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -3244,16 +3156,16 @@
         <v>151</v>
       </c>
       <c r="K26" t="n">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="L26" t="n">
-        <v>55.5</v>
+        <v>61.5</v>
       </c>
       <c r="M26" t="n">
         <v>0.5</v>
       </c>
       <c r="N26" t="n">
-        <v>1.01</v>
+        <v>2.78</v>
       </c>
       <c r="O26" t="inlineStr">
         <is>
@@ -3364,16 +3276,16 @@
         <v>268</v>
       </c>
       <c r="K28" t="n">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="L28" t="n">
-        <v>33.5</v>
+        <v>41.5</v>
       </c>
       <c r="M28" t="n">
         <v>0.5</v>
       </c>
       <c r="N28" t="n">
-        <v>1.27</v>
+        <v>0.96</v>
       </c>
       <c r="O28" t="inlineStr">
         <is>
@@ -3424,16 +3336,16 @@
         <v>473</v>
       </c>
       <c r="K29" t="n">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="L29" t="n">
-        <v>171.5</v>
+        <v>180.5</v>
       </c>
       <c r="M29" t="n">
         <v>0.5</v>
       </c>
       <c r="N29" t="n">
-        <v>1.33</v>
+        <v>1.46</v>
       </c>
       <c r="O29" t="inlineStr">
         <is>
@@ -3488,16 +3400,16 @@
         <v>205</v>
       </c>
       <c r="K30" t="n">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="L30" t="n">
-        <v>76.5</v>
+        <v>89.5</v>
       </c>
       <c r="M30" t="n">
         <v>0.5</v>
       </c>
       <c r="N30" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="O30" t="inlineStr">
         <is>
@@ -3612,16 +3524,16 @@
         <v>190</v>
       </c>
       <c r="K32" t="n">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="L32" t="n">
-        <v>9.5</v>
+        <v>28</v>
       </c>
       <c r="M32" t="n">
         <v>0.5</v>
       </c>
       <c r="N32" t="n">
-        <v>0.85</v>
+        <v>0.54</v>
       </c>
       <c r="O32" t="inlineStr">
         <is>
@@ -3676,16 +3588,16 @@
         <v>555</v>
       </c>
       <c r="K33" t="n">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="L33" t="n">
-        <v>143.5</v>
+        <v>152</v>
       </c>
       <c r="M33" t="n">
         <v>0.5</v>
       </c>
       <c r="N33" t="n">
-        <v>1.61</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O33" t="inlineStr">
         <is>
@@ -3749,7 +3661,7 @@
         <v>0.5</v>
       </c>
       <c r="N34" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O34" t="inlineStr">
         <is>
@@ -3804,20 +3716,20 @@
         <v>355</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M35" t="n">
         <v>0.5</v>
       </c>
       <c r="N35" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
+          <t>PARCIAL (limitado tela)</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
@@ -3868,16 +3780,16 @@
         <v>124</v>
       </c>
       <c r="K36" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="L36" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="M36" t="n">
         <v>0.5</v>
       </c>
       <c r="N36" t="n">
-        <v>1.35</v>
+        <v>1.7</v>
       </c>
       <c r="O36" t="inlineStr">
         <is>
@@ -3928,20 +3840,20 @@
         <v>135</v>
       </c>
       <c r="K37" t="n">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="L37" t="n">
-        <v>49.6</v>
+        <v>54</v>
       </c>
       <c r="M37" t="n">
         <v>0.4</v>
       </c>
       <c r="N37" t="n">
-        <v>1.01</v>
+        <v>2.78</v>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>PARCIAL (limitado tela)</t>
+          <t>OK</t>
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
@@ -4048,16 +3960,16 @@
         <v>232</v>
       </c>
       <c r="K39" t="n">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="L39" t="n">
-        <v>28.8</v>
+        <v>35.6</v>
       </c>
       <c r="M39" t="n">
         <v>0.4</v>
       </c>
       <c r="N39" t="n">
-        <v>1.27</v>
+        <v>0.96</v>
       </c>
       <c r="O39" t="inlineStr">
         <is>
@@ -4108,16 +4020,16 @@
         <v>357</v>
       </c>
       <c r="K40" t="n">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="L40" t="n">
-        <v>129.2</v>
+        <v>136.4</v>
       </c>
       <c r="M40" t="n">
         <v>0.4</v>
       </c>
       <c r="N40" t="n">
-        <v>1.33</v>
+        <v>1.46</v>
       </c>
       <c r="O40" t="inlineStr">
         <is>
@@ -4232,16 +4144,16 @@
         <v>193</v>
       </c>
       <c r="K42" t="n">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="L42" t="n">
-        <v>37.6</v>
+        <v>50</v>
       </c>
       <c r="M42" t="n">
         <v>0.4</v>
       </c>
       <c r="N42" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="O42" t="inlineStr">
         <is>
@@ -4292,16 +4204,16 @@
         <v>417</v>
       </c>
       <c r="K43" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="L43" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="M43" t="n">
         <v>0.4</v>
       </c>
       <c r="N43" t="n">
-        <v>1.61</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O43" t="inlineStr">
         <is>
@@ -4425,7 +4337,7 @@
         <v>0.4</v>
       </c>
       <c r="N45" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O45" t="inlineStr">
         <is>
@@ -4489,7 +4401,7 @@
         <v>0.4</v>
       </c>
       <c r="N46" t="n">
-        <v>0.71</v>
+        <v>0.02</v>
       </c>
       <c r="O46" t="inlineStr">
         <is>
@@ -4498,7 +4410,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>Stock crítico — excluir o esperar compra</t>
+          <t>Limitado por tela disponible</t>
         </is>
       </c>
     </row>
@@ -4544,20 +4456,20 @@
         <v>272</v>
       </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L47" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="M47" t="n">
         <v>0.4</v>
       </c>
       <c r="N47" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
+          <t>PARCIAL (limitado tela)</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -4608,16 +4520,16 @@
         <v>162</v>
       </c>
       <c r="K48" t="n">
-        <v>92</v>
+        <v>112</v>
       </c>
       <c r="L48" t="n">
-        <v>36.8</v>
+        <v>44.8</v>
       </c>
       <c r="M48" t="n">
         <v>0.4</v>
       </c>
       <c r="N48" t="n">
-        <v>1.35</v>
+        <v>1.7</v>
       </c>
       <c r="O48" t="inlineStr">
         <is>
@@ -4668,16 +4580,16 @@
         <v>154</v>
       </c>
       <c r="K49" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="L49" t="n">
-        <v>56.1</v>
+        <v>62.7</v>
       </c>
       <c r="M49" t="n">
         <v>0.66</v>
       </c>
       <c r="N49" t="n">
-        <v>1.01</v>
+        <v>2.78</v>
       </c>
       <c r="O49" t="inlineStr">
         <is>
@@ -4788,16 +4700,16 @@
         <v>267</v>
       </c>
       <c r="K51" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="L51" t="n">
-        <v>33</v>
+        <v>40.92</v>
       </c>
       <c r="M51" t="n">
         <v>0.66</v>
       </c>
       <c r="N51" t="n">
-        <v>1.27</v>
+        <v>0.96</v>
       </c>
       <c r="O51" t="inlineStr">
         <is>
@@ -4848,16 +4760,16 @@
         <v>336</v>
       </c>
       <c r="K52" t="n">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="L52" t="n">
-        <v>121.44</v>
+        <v>128.04</v>
       </c>
       <c r="M52" t="n">
         <v>0.66</v>
       </c>
       <c r="N52" t="n">
-        <v>1.33</v>
+        <v>1.46</v>
       </c>
       <c r="O52" t="inlineStr">
         <is>
@@ -4912,16 +4824,16 @@
         <v>277</v>
       </c>
       <c r="K53" t="n">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="L53" t="n">
-        <v>103.62</v>
+        <v>121.44</v>
       </c>
       <c r="M53" t="n">
         <v>0.66</v>
       </c>
       <c r="N53" t="n">
-        <v>0.61</v>
+        <v>0.52</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
@@ -5036,16 +4948,16 @@
         <v>133</v>
       </c>
       <c r="K55" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="L55" t="n">
-        <v>6.6</v>
+        <v>19.14</v>
       </c>
       <c r="M55" t="n">
         <v>0.66</v>
       </c>
       <c r="N55" t="n">
-        <v>0.85</v>
+        <v>0.54</v>
       </c>
       <c r="O55" t="inlineStr">
         <is>
@@ -5100,16 +5012,16 @@
         <v>557</v>
       </c>
       <c r="K56" t="n">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="L56" t="n">
-        <v>143.88</v>
+        <v>152.46</v>
       </c>
       <c r="M56" t="n">
         <v>0.66</v>
       </c>
       <c r="N56" t="n">
-        <v>1.61</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O56" t="inlineStr">
         <is>
@@ -5173,7 +5085,7 @@
         <v>0.66</v>
       </c>
       <c r="N57" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O57" t="inlineStr">
         <is>
@@ -5228,20 +5140,20 @@
         <v>245</v>
       </c>
       <c r="K58" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L58" t="n">
-        <v>0</v>
+        <v>1.32</v>
       </c>
       <c r="M58" t="n">
         <v>0.66</v>
       </c>
       <c r="N58" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
+          <t>PARCIAL (limitado tela)</t>
         </is>
       </c>
       <c r="P58" t="inlineStr">
@@ -5292,16 +5204,16 @@
         <v>183</v>
       </c>
       <c r="K59" t="n">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="L59" t="n">
-        <v>41.58</v>
+        <v>50.16</v>
       </c>
       <c r="M59" t="n">
         <v>0.66</v>
       </c>
       <c r="N59" t="n">
-        <v>1.35</v>
+        <v>1.7</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
@@ -5352,16 +5264,16 @@
         <v>286</v>
       </c>
       <c r="K60" t="n">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="L60" t="n">
-        <v>105.04</v>
+        <v>117</v>
       </c>
       <c r="M60" t="n">
         <v>0.52</v>
       </c>
       <c r="N60" t="n">
-        <v>1.01</v>
+        <v>2.78</v>
       </c>
       <c r="O60" t="inlineStr">
         <is>
@@ -5472,16 +5384,16 @@
         <v>269</v>
       </c>
       <c r="K62" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="L62" t="n">
-        <v>33.28</v>
+        <v>41.6</v>
       </c>
       <c r="M62" t="n">
         <v>0.52</v>
       </c>
       <c r="N62" t="n">
-        <v>1.27</v>
+        <v>0.96</v>
       </c>
       <c r="O62" t="inlineStr">
         <is>
@@ -5532,16 +5444,16 @@
         <v>388</v>
       </c>
       <c r="K63" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="L63" t="n">
-        <v>140.4</v>
+        <v>148.2</v>
       </c>
       <c r="M63" t="n">
         <v>0.52</v>
       </c>
       <c r="N63" t="n">
-        <v>1.33</v>
+        <v>1.46</v>
       </c>
       <c r="O63" t="inlineStr">
         <is>
@@ -5660,16 +5572,16 @@
         <v>283</v>
       </c>
       <c r="K65" t="n">
-        <v>106</v>
+        <v>141</v>
       </c>
       <c r="L65" t="n">
-        <v>55.12</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="M65" t="n">
         <v>0.52</v>
       </c>
       <c r="N65" t="n">
-        <v>0.53</v>
+        <v>0.66</v>
       </c>
       <c r="O65" t="inlineStr">
         <is>
@@ -5720,16 +5632,16 @@
         <v>561</v>
       </c>
       <c r="K66" t="n">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="L66" t="n">
-        <v>145.08</v>
+        <v>153.4</v>
       </c>
       <c r="M66" t="n">
         <v>0.52</v>
       </c>
       <c r="N66" t="n">
-        <v>1.61</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O66" t="inlineStr">
         <is>
@@ -5853,7 +5765,7 @@
         <v>0.52</v>
       </c>
       <c r="N68" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="O68" t="inlineStr">
         <is>
@@ -5917,7 +5829,7 @@
         <v>0.52</v>
       </c>
       <c r="N69" t="n">
-        <v>0.71</v>
+        <v>0.02</v>
       </c>
       <c r="O69" t="inlineStr">
         <is>
@@ -5926,7 +5838,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>Stock crítico — excluir o esperar compra</t>
+          <t>Limitado por tela disponible</t>
         </is>
       </c>
     </row>
@@ -5972,20 +5884,20 @@
         <v>146</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L70" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="M70" t="n">
         <v>0.52</v>
       </c>
       <c r="N70" t="n">
-        <v>1.77</v>
+        <v>1.14</v>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>SIN TELA</t>
+          <t>PARCIAL (limitado tela)</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
@@ -6036,16 +5948,16 @@
         <v>163</v>
       </c>
       <c r="K71" t="n">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="L71" t="n">
-        <v>36.92</v>
+        <v>44.72</v>
       </c>
       <c r="M71" t="n">
         <v>0.52</v>
       </c>
       <c r="N71" t="n">
-        <v>1.35</v>
+        <v>1.7</v>
       </c>
       <c r="O71" t="inlineStr">
         <is>
@@ -6070,10 +5982,10 @@
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="n">
-        <v>6124</v>
+        <v>6797</v>
       </c>
       <c r="L72" t="n">
-        <v>2670.02</v>
+        <v>2977.64</v>
       </c>
     </row>
   </sheetData>
@@ -6161,7 +6073,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>659.17</v>
+        <v>689.9</v>
       </c>
       <c r="C2" t="n">
         <v>145</v>
@@ -6170,19 +6082,19 @@
         <v>180</v>
       </c>
       <c r="E2" t="n">
-        <v>343</v>
+        <v>361</v>
       </c>
       <c r="F2" t="n">
-        <v>323</v>
+        <v>341</v>
       </c>
       <c r="G2" t="n">
-        <v>184</v>
+        <v>194</v>
       </c>
       <c r="H2" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="I2" t="n">
-        <v>1445</v>
+        <v>1506</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -6197,7 +6109,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>626.4299999999999</v>
+        <v>657.16</v>
       </c>
       <c r="C3" t="n">
         <v>130</v>
@@ -6206,19 +6118,19 @@
         <v>158</v>
       </c>
       <c r="E3" t="n">
-        <v>287</v>
+        <v>304</v>
       </c>
       <c r="F3" t="n">
-        <v>270</v>
+        <v>285</v>
       </c>
       <c r="G3" t="n">
-        <v>218</v>
+        <v>231</v>
       </c>
       <c r="H3" t="n">
-        <v>279</v>
+        <v>295</v>
       </c>
       <c r="I3" t="n">
-        <v>1342</v>
+        <v>1403</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -6233,7 +6145,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>317.61</v>
+        <v>348.34</v>
       </c>
       <c r="C4" t="n">
         <v>62</v>
@@ -6242,19 +6154,19 @@
         <v>107</v>
       </c>
       <c r="E4" t="n">
-        <v>111</v>
+        <v>123</v>
       </c>
       <c r="F4" t="n">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="G4" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H4" t="n">
-        <v>202</v>
+        <v>225</v>
       </c>
       <c r="I4" t="n">
-        <v>691</v>
+        <v>747</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -6269,7 +6181,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>240.73</v>
+        <v>271.46</v>
       </c>
       <c r="C5" t="n">
         <v>56</v>
@@ -6278,19 +6190,19 @@
         <v>142</v>
       </c>
       <c r="E5" t="n">
-        <v>153</v>
+        <v>179</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>157</v>
+        <v>184</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>508</v>
+        <v>561</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -6305,7 +6217,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>190.27</v>
+        <v>221</v>
       </c>
       <c r="C6" t="n">
         <v>17</v>
@@ -6314,19 +6226,19 @@
         <v>175</v>
       </c>
       <c r="E6" t="n">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="F6" t="n">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="G6" t="n">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="H6" t="n">
-        <v>64</v>
+        <v>80</v>
       </c>
       <c r="I6" t="n">
-        <v>445</v>
+        <v>506</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -6337,32 +6249,32 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Blanco</t>
+          <t>Lila</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>162.04</v>
+        <v>188.44</v>
       </c>
       <c r="C7" t="n">
-        <v>230</v>
+        <v>67</v>
       </c>
       <c r="D7" t="n">
-        <v>112</v>
+        <v>147</v>
       </c>
       <c r="E7" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>44</v>
+        <v>125</v>
       </c>
       <c r="G7" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>29</v>
+        <v>141</v>
       </c>
       <c r="I7" t="n">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -6373,32 +6285,32 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lila</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>157.71</v>
+        <v>175.38</v>
       </c>
       <c r="C8" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="D8" t="n">
-        <v>147</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="F8" t="n">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="H8" t="n">
-        <v>106</v>
+        <v>86</v>
       </c>
       <c r="I8" t="n">
-        <v>414</v>
+        <v>342</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -6409,32 +6321,32 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Vinotinto</t>
+          <t>Blanco</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>144.65</v>
+        <v>162.04</v>
       </c>
       <c r="C9" t="n">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="E9" t="n">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="F9" t="n">
-        <v>92</v>
+        <v>44</v>
       </c>
       <c r="G9" t="n">
-        <v>63</v>
+        <v>24</v>
       </c>
       <c r="H9" t="n">
-        <v>71</v>
+        <v>29</v>
       </c>
       <c r="I9" t="n">
-        <v>282</v>
+        <v>473</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -6445,32 +6357,32 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Morado</t>
+          <t>Púrpura</t>
         </is>
       </c>
       <c r="B10" t="n">
         <v>94.2</v>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>106</v>
       </c>
       <c r="E10" t="n">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -6481,32 +6393,32 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Púrpura</t>
+          <t>Morado</t>
         </is>
       </c>
       <c r="B11" t="n">
         <v>94.2</v>
       </c>
       <c r="C11" t="n">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>106</v>
+        <v>0</v>
       </c>
       <c r="E11" t="n">
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>278</v>
+        <v>0</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -6557,7 +6469,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>16.95</v>
+        <v>47.68</v>
       </c>
       <c r="C13" t="n">
         <v>0</v>
@@ -6566,19 +6478,19 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
       </c>
       <c r="I13" t="n">
-        <v>29</v>
+        <v>85</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -6593,28 +6505,28 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15.29</v>
+        <v>46.02</v>
       </c>
       <c r="C14" t="n">
         <v>52</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="E14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
-        <v>52</v>
+        <v>144</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -6629,13 +6541,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.71</v>
+        <v>31.44</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E15" t="n">
         <v>0</v>
@@ -6650,11 +6562,11 @@
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>NO PRODUCIR — sin tela</t>
+          <t>Solo KIDS parcial</t>
         </is>
       </c>
     </row>
@@ -6665,7 +6577,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0</v>
+        <v>0.18</v>
       </c>
       <c r="C16" t="n">
         <v>0</v>

</xml_diff>